<commit_message>
Anlagenzustandsanalyse: Zielwert technische Verfügbarkeit 92 % bestätigt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012JbEhcYgieDunoMLuHo6SL
</commit_message>
<xml_diff>
--- a/Anlagenzustandsanalyse.xlsx
+++ b/Anlagenzustandsanalyse.xlsx
@@ -20560,7 +20560,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Annahme: 92 % wie im Vorlage-Punkt 24 der Datei „2026_Audit_Instandhaltung_Allgemein“ (dort Hinweis 90 % / 80 %). Bitte gültigen Zielwert bestätigen.</t>
+          <t>Zielwert 92 % – vom Auftraggeber bestätigt (entspricht Vorlage-Punkt 24 der Datei „2026_Audit_Instandhaltung_Allgemein“).</t>
         </is>
       </c>
       <c r="E11" s="1" t="n"/>
@@ -22112,12 +22112,12 @@
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="78" t="inlineStr">
         <is>
-          <t>Offene Punkte / Annahmen</t>
+          <t>Zielwerte und Annahmen</t>
         </is>
       </c>
       <c r="B46" s="1" t="n"/>
     </row>
-    <row r="47" ht="27" customHeight="1">
+    <row r="47" ht="13.5" customHeight="1">
       <c r="A47" s="90" t="inlineStr">
         <is>
           <t>Ziel Verfügbarkeit</t>
@@ -22125,7 +22125,7 @@
       </c>
       <c r="B47" s="91" t="inlineStr">
         <is>
-          <t>92 % aus Vorlage-Punkt 24 der Datei „2026_Audit_Instandhaltung_Allgemein“ übernommen; dort ist der Wert zwischen deutscher und englischer Fassung uneinheitlich. Bitte bestätigen (Blatt „Einstellungen“).</t>
+          <t>92 % – bestätigt. Wert im Blatt „Einstellungen“ änderbar.</t>
         </is>
       </c>
     </row>

</xml_diff>